<commit_message>
Keep Anna on Playables Excel and hide pay hours from everyone but DL.
Writing Сергій as MOTION at column E shifted 2DART 1, so ingest dropped Anna's hours. Excel now binds AD/DEV to the live sheet columns, restores SP_PLBL_check.xlsx from Drive, and PLAYABLE HOURS (producer, LP $7, buffer) is finance-only.

Co-authored-by: lisenbart <lisenbart@gmail.com>
</commit_message>
<xml_diff>
--- a/data/SP_PLBL_check.xlsx
+++ b/data/SP_PLBL_check.xlsx
@@ -95,7 +95,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -145,6 +145,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C9A0DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="007ED4C2"/>
       </patternFill>
     </fill>
@@ -180,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -262,6 +267,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -347,20 +355,15 @@
   <commentList>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>lg-id:designer3</t>
+        <t>lg-id:artdir1</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>lg-id:artdir1</t>
+        <t>lg-id:artdir2</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>lg-id:artdir2</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>lg-id:programmer1</t>
       </text>
@@ -592,20 +595,15 @@
       </c>
       <c r="E1" s="33" t="inlineStr">
         <is>
-          <t>Сергій</t>
+          <t>Анна</t>
         </is>
       </c>
       <c r="F1" s="33" t="inlineStr">
         <is>
-          <t>Анна</t>
+          <t>Юля</t>
         </is>
       </c>
       <c r="G1" s="33" t="inlineStr">
-        <is>
-          <t>Юля</t>
-        </is>
-      </c>
-      <c r="H1" s="33" t="inlineStr">
         <is>
           <t>Богдан</t>
         </is>
@@ -634,20 +632,15 @@
       </c>
       <c r="E2" s="35" t="inlineStr">
         <is>
-          <t>MOTION</t>
+          <t>2DART 1</t>
         </is>
       </c>
       <c r="F2" s="35" t="inlineStr">
         <is>
-          <t>2DART 1</t>
+          <t>2DART 2</t>
         </is>
       </c>
       <c r="G2" s="35" t="inlineStr">
-        <is>
-          <t>2DART 2</t>
-        </is>
-      </c>
-      <c r="H2" s="35" t="inlineStr">
         <is>
           <t>PRGMM1</t>
         </is>
@@ -698,15 +691,16 @@
         <v>26</v>
       </c>
       <c r="D6" s="38">
-        <f>SUM(E6:H6)</f>
-        <v/>
-      </c>
-      <c r="E6" s="38" t="n"/>
-      <c r="F6" s="38" t="n"/>
-      <c r="G6" s="39" t="n">
+        <f>SUM(E6:G6)</f>
+        <v/>
+      </c>
+      <c r="E6" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="40" t="n">
         <v>8</v>
       </c>
-      <c r="H6" s="40" t="n">
+      <c r="G6" s="41" t="n">
         <v>16</v>
       </c>
     </row>
@@ -747,13 +741,14 @@
         <v>30</v>
       </c>
       <c r="D9" s="38">
-        <f>SUM(E9:H9)</f>
-        <v/>
-      </c>
-      <c r="E9" s="38" t="n"/>
+        <f>SUM(E9:G9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="39" t="n">
+        <v>9</v>
+      </c>
       <c r="F9" s="38" t="n"/>
-      <c r="G9" s="38" t="n"/>
-      <c r="H9" s="40" t="n">
+      <c r="G9" s="41" t="n">
         <v>20</v>
       </c>
     </row>
@@ -768,13 +763,12 @@
         <v>5</v>
       </c>
       <c r="D10" s="38">
-        <f>SUM(E10:H10)</f>
+        <f>SUM(E10:G10)</f>
         <v/>
       </c>
       <c r="E10" s="38" t="n"/>
       <c r="F10" s="38" t="n"/>
-      <c r="G10" s="38" t="n"/>
-      <c r="H10" s="40" t="n">
+      <c r="G10" s="41" t="n">
         <v>4</v>
       </c>
     </row>
@@ -789,15 +783,16 @@
         <v>26</v>
       </c>
       <c r="D11" s="38">
-        <f>SUM(E11:H11)</f>
-        <v/>
-      </c>
-      <c r="E11" s="38" t="n"/>
-      <c r="F11" s="38" t="n"/>
-      <c r="G11" s="39" t="n">
+        <f>SUM(E11:G11)</f>
+        <v/>
+      </c>
+      <c r="E11" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="40" t="n">
         <v>8</v>
       </c>
-      <c r="H11" s="40" t="n">
+      <c r="G11" s="41" t="n">
         <v>16</v>
       </c>
     </row>
@@ -812,13 +807,14 @@
         <v>28</v>
       </c>
       <c r="D12" s="38">
-        <f>SUM(E12:H12)</f>
-        <v/>
-      </c>
-      <c r="E12" s="38" t="n"/>
+        <f>SUM(E12:G12)</f>
+        <v/>
+      </c>
+      <c r="E12" s="39" t="n">
+        <v>11</v>
+      </c>
       <c r="F12" s="38" t="n"/>
-      <c r="G12" s="38" t="n"/>
-      <c r="H12" s="40" t="n">
+      <c r="G12" s="41" t="n">
         <v>16</v>
       </c>
     </row>
@@ -833,13 +829,14 @@
         <v>27</v>
       </c>
       <c r="D13" s="38">
-        <f>SUM(E13:H13)</f>
-        <v/>
-      </c>
-      <c r="E13" s="38" t="n"/>
+        <f>SUM(E13:G13)</f>
+        <v/>
+      </c>
+      <c r="E13" s="39" t="n">
+        <v>8</v>
+      </c>
       <c r="F13" s="38" t="n"/>
-      <c r="G13" s="38" t="n"/>
-      <c r="H13" s="40" t="n">
+      <c r="G13" s="41" t="n">
         <v>18</v>
       </c>
     </row>
@@ -854,15 +851,16 @@
         <v>30</v>
       </c>
       <c r="D14" s="38">
-        <f>SUM(E14:H14)</f>
-        <v/>
-      </c>
-      <c r="E14" s="38" t="n"/>
-      <c r="F14" s="38" t="n"/>
-      <c r="G14" s="39" t="n">
+        <f>SUM(E14:G14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="H14" s="40" t="n">
+      <c r="G14" s="41" t="n">
         <v>18</v>
       </c>
     </row>

</xml_diff>